<commit_message>
chore: run 2026-04-20 09:39 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_20_04_2026.xlsx
+++ b/logs/Consolidado_20_04_2026.xlsx
@@ -620,7 +620,7 @@
         <v>152</v>
       </c>
       <c r="C2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -677,13 +677,13 @@
         <v>69</v>
       </c>
       <c r="C5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -3264,40 +3264,40 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="7" t="inlineStr">
-        <is>
-          <t>20/04/2026</t>
-        </is>
-      </c>
-      <c r="B63" s="7" t="inlineStr">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>20/04/2026</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C63" s="7" t="inlineStr">
+      <c r="C63" s="5" t="inlineStr">
         <is>
           <t>Hyaluron Activ B3 Cell Renewal Aqua Cream-Gel
 Creme-Gel Dia Rugas AH, Niacinamida
 50 ml</t>
         </is>
       </c>
-      <c r="D63" s="7" t="inlineStr">
+      <c r="D63" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/hyaluron-activ-b3-cell-renewal-aqua-cream-gel-7982205.html</t>
         </is>
       </c>
-      <c r="E63" s="7" t="inlineStr"/>
-      <c r="F63" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G63" s="7" t="inlineStr">
+      <c r="E63" s="5" t="inlineStr"/>
+      <c r="F63" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G63" s="5" t="inlineStr">
         <is>
           <t>7982205</t>
         </is>
       </c>
-      <c r="H63" s="7" t="inlineStr">
+      <c r="H63" s="5" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -11777,7 +11777,9 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Bad gateway Error code 502</t>
+          <t>Okara Silver Toning Shampoo
+Champô Violeta Cabelo Branco Grisalho ou Louro
+200 ml</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -11791,10 +11793,14 @@
           <t>In Stock</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr"/>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>6759950</t>
+        </is>
+      </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>Sem desconto</t>
+          <t>25%</t>
         </is>
       </c>
     </row>
@@ -12319,40 +12325,40 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="7" t="inlineStr">
-        <is>
-          <t>20/04/2026</t>
-        </is>
-      </c>
-      <c r="B51" s="7" t="inlineStr">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>20/04/2026</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C51" s="7" t="inlineStr">
+      <c r="C51" s="3" t="inlineStr">
         <is>
           <t>Sublime Curl nutri-Activating Cream
 Creme Cabelo Leave-In Redefinidor de Caracóis
 100 ml</t>
         </is>
       </c>
-      <c r="D51" s="7" t="inlineStr">
+      <c r="D51" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/sublime-curl-nutri-activating-cream-5972165.html</t>
         </is>
       </c>
-      <c r="E51" s="7" t="inlineStr"/>
-      <c r="F51" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G51" s="7" t="inlineStr">
+      <c r="E51" s="3" t="inlineStr"/>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
         <is>
           <t>5972165</t>
         </is>
       </c>
-      <c r="H51" s="7" t="inlineStr">
+      <c r="H51" s="3" t="inlineStr">
         <is>
           <t>28%</t>
         </is>

</xml_diff>